<commit_message>
Tracker: Epic 6 Sprint 21 - My Work task management (ASK-28 + ASK-29); Master Tracker updated
Epic 6 Backlog U7-21.1..15: New Task form, Asked by me, Waiting for my
approval, My team, links that land, approval moment, phone pass, who is on a
task, stages and flags, task access, who may change a task, stuck work reaches
the manager first, safe testing (13 Done, each with its commit and checks);
open: Flutter app parity, separate test database. UI Redesign Log +11 commits,
Dashboard and Cover rows for Sprint 21. Master Tracker: Epic 6 130/217 (60%),
all epics 562/817 (69%).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +99,10 @@
       <i val="1"/>
       <color rgb="00666666"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -169,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +230,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1450,6 +1457,49 @@
       <c r="B103" t="inlineStr">
         <is>
           <t>Backlog</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>Sprint 21 -- My Work - task management</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MyWork.js, Tasks.js, lib/taskAccess.js, routers/tasks.py, routers/desk.py, services/tasks.py, services/finance_signals.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Founder plan 2026-09-14: everyone sees the work they are part of, clear people and stages on a task, approval as a step, access rules, and stuck work that climbs to the manager before the owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>In progress -- 13 of 15 Done; open: Flutter app parity, separate test database</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1493,7 +1543,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 64 of 153 items Done  (42%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.</t>
+          <t>Epic 6 progress: 64 of 153 items Done  (42%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 13 of 15 Done.</t>
         </is>
       </c>
     </row>
@@ -2191,6 +2241,39 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>See 'UI Redesign Log' sheet — 105 karma / RD / NM / MPWA UI commits, all shipped to Backend_optimization. Sprint 19 carries the KM-* / KR-14.2-24 mobile pass entries in Backlog to keep the totals clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sprint 21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>My Work - task management</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>13</v>
+      </c>
+      <c r="D26" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Task management plan (docs/TASK_MANAGEMENT_PLAN.md), ASK-28 + ASK-29, 2026-09-14/15: New Task form, Asked by me / Waiting for my approval / My team views, links that land, approval moment, who is on a task, stages and flags, task access, who may change a task, stuck work reaches the manager first. Open: Flutter app, separate test database.</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4983,6 +5066,303 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>9b88efc</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr">
+        <is>
+          <t>ASK-29 - New Task form: what, department, who, when; the rest under More options</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>72e0598</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-01 - Asked by me view</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>b1c9daf</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-02 - Waiting for my approval (Approvals view + Desk card)</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>8eac435</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-03 - My team for managers</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>ae6675d</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-05 - approval before work starts or before it is marked done</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>564732d</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-04 - task links always land; every view is an address</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>009bd2d</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 - phone pass, approver check, real-save journeys, old audit scripts made safe</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>93686c2</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-06 - who is on a task: Doer, Helpers, Asked by, Approver</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>abe4b40</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-07 - stages and flags: To do / Doing / Done, Waiting on someone</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>b2ae273</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-08 - task access: who may assign, who sees all tasks</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>92c3d0f</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>ASK-28 item 7 + Phase 7 - who may change a task; stuck work reaches the manager first</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4994,7 +5374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15251,6 +15631,846 @@
       <c r="L181" t="inlineStr">
         <is>
           <t>Epic 3 (moved 2026-09-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.1</t>
+        </is>
+      </c>
+      <c r="B182" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, Tasks.js (NewTaskDialog)</t>
+        </is>
+      </c>
+      <c r="C182" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D182" s="28" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+      <c r="E182" s="28" t="inlineStr">
+        <is>
+          <t>New Task form -- what, department, who, when; the rest under More options</t>
+        </is>
+      </c>
+      <c r="F182" s="28" t="inlineStr">
+        <is>
+          <t>ASK-29 / plan Phase 5. Quick add: title with an inline error, Department, one Assign to (a person, or a team routed to its least busy member), due presets No date / Today / Tomorrow / In a week / Pick a date. More options: priority, helpers, description, due time, expected result, approval + approver + when, proof, reference files. Operational category and Supporting employee dropped from the form. Due Today no longer reads Overdue the same morning.</t>
+        </is>
+      </c>
+      <c r="G182" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H182" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I182" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J182" s="28" t="n"/>
+      <c r="K182" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 9b88efc (2026-09-14). Glass pass 0eaa411 moved it onto GlassSelect. Acceptance ux_newtask_form_0914.py re-run green through TK-08.</t>
+        </is>
+      </c>
+      <c r="L182" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.2</t>
+        </is>
+      </c>
+      <c r="B183" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, services/tasks.py</t>
+        </is>
+      </c>
+      <c r="C183" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D183" s="28" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="E183" s="28" t="inlineStr">
+        <is>
+          <t>Asked by me -- see the work you handed to other people</t>
+        </is>
+      </c>
+      <c r="F183" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-01 / plan 1.1. GET /tasks?view=asked (tasks I created that are not mine to do) + an Asked by me view in the switcher, kept in ?view=, with Department / Person / Status filters and its own empty state. The person who asked may leave a note.</t>
+        </is>
+      </c>
+      <c r="G183" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H183" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I183" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J183" s="28" t="n"/>
+      <c r="K183" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 72e0598 (2026-09-14). Real-save journey test_asked_by_me_non_owner_keeps_sight_of_work_they_hand_out; browser 20/20 writes blocked.</t>
+        </is>
+      </c>
+      <c r="L183" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.3</t>
+        </is>
+      </c>
+      <c r="B184" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, Desk.js, services/tasks.py</t>
+        </is>
+      </c>
+      <c r="C184" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D184" s="28" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="E184" s="28" t="inlineStr">
+        <is>
+          <t>Waiting for my approval -- every approver sees what waits on them</t>
+        </is>
+      </c>
+      <c r="F184" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-02 / plan 1.2 + 1.5. GET /tasks?view=approvals (the owner all; a named approver their own; an approvals holder also the unnamed ones). Feeds the Approvals view in My Work (with its count) and the Decision Desk Task approvals card. Approval notifications open the task in Approvals.</t>
+        </is>
+      </c>
+      <c r="G184" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H184" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I184" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J184" s="28" t="n"/>
+      <c r="K184" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED b1c9daf (2026-09-14). Real-save journey with a non-owner named approver; browser checks owner 7/7 vs API.</t>
+        </is>
+      </c>
+      <c r="L184" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.4</t>
+        </is>
+      </c>
+      <c r="B185" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, services/tasks.py</t>
+        </is>
+      </c>
+      <c r="C185" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D185" s="28" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="E185" s="28" t="inlineStr">
+        <is>
+          <t>My team -- a manager sees the work of the people who report to them</t>
+        </is>
+      </c>
+      <c r="F185" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-03 / plan 1.3 (D3). GET /tasks?view=team through the Reporting Manager field (direct reports, as doer or helper). Shown to a non-owner with reports; the owner keeps All Tasks. The manager opens a report's task, its activity, and notes on it.</t>
+        </is>
+      </c>
+      <c r="G185" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H185" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I185" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J185" s="28" t="n"/>
+      <c r="K185" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 8eac435 (2026-09-14). Real data (Sunita Rao manages sai) 21/21 writes blocked; real-save journey test_my_team_manager_sees_opens_and_notes_on_reports_work.</t>
+        </is>
+      </c>
+      <c r="L185" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.5</t>
+        </is>
+      </c>
+      <c r="B186" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js</t>
+        </is>
+      </c>
+      <c r="C186" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D186" s="28" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="E186" s="28" t="inlineStr">
+        <is>
+          <t>Links always land -- a task link opens its task, and every view is an address</t>
+        </is>
+      </c>
+      <c r="F186" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-04 / plan 1.4. /my-work?task=&lt;id&gt; (and ?focus=task:&lt;id&gt;) opens the drawer whatever the view, from the single-task request when the task is not in the list; missing and refused tasks say so. Every view lives in ?view= and survives refresh, Back and Forward.</t>
+        </is>
+      </c>
+      <c r="G186" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H186" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I186" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J186" s="28" t="n"/>
+      <c r="K186" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 564732d + tracker 7aa4031 (2026-09-14). Acceptance ux_task_links_0914.py 23/23 on real data, writes blocked.</t>
+        </is>
+      </c>
+      <c r="L186" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.6</t>
+        </is>
+      </c>
+      <c r="B187" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, routers/tasks.py</t>
+        </is>
+      </c>
+      <c r="C187" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D187" s="28" t="inlineStr">
+        <is>
+          <t>Approval</t>
+        </is>
+      </c>
+      <c r="E187" s="28" t="inlineStr">
+        <is>
+          <t>Approval moment -- before work starts, or before it is marked done</t>
+        </is>
+      </c>
+      <c r="F187" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-05 / plan Phase 4 (D2). The creator picks per task. Before closing: Complete sends it to the approver (Under review), Approve closes it, Request changes returns it with the reason. The server checks the named approver can actually approve (4.3). Cards say Approval to start / Approval to close.</t>
+        </is>
+      </c>
+      <c r="G187" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H187" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I187" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J187" s="28" t="n"/>
+      <c r="K187" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED ae6675d; approver check in 009bd2d (2026-09-14). 17 unit tests; real-save journeys for both moments; browser 19/19.</t>
+        </is>
+      </c>
+      <c r="L187" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.7</t>
+        </is>
+      </c>
+      <c r="B188" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, Tasks.js (phone)</t>
+        </is>
+      </c>
+      <c r="C188" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D188" s="28" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E188" s="28" t="inlineStr">
+        <is>
+          <t>Phone pass -- New Task and every My Work view on a phone</t>
+        </is>
+      </c>
+      <c r="F188" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 / plan 5.4. New Task as a full-screen sheet with Create in reach; one view pill opening a sheet of the person's views (My Tasks, Asked by me, My team, All Tasks, Approvals with its count). Checked at 390x844. Later (8fbe532, Chinmay) the task itself opens full screen on a phone.</t>
+        </is>
+      </c>
+      <c r="G188" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H188" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I188" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J188" s="28" t="n"/>
+      <c r="K188" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 009bd2d (2026-09-14). ux_task_phone_0914.py 21/21, re-run green after the full-screen change.</t>
+        </is>
+      </c>
+      <c r="L188" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.8</t>
+        </is>
+      </c>
+      <c r="B189" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, routers/tasks.py, mobile/work_screen.dart</t>
+        </is>
+      </c>
+      <c r="C189" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D189" s="28" t="inlineStr">
+        <is>
+          <t>Data model</t>
+        </is>
+      </c>
+      <c r="E189" s="28" t="inlineStr">
+        <is>
+          <t>Who is on a task -- Doer, Helpers, Asked by, Approver</t>
+        </is>
+      </c>
+      <c r="F189" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-06 / plan Phase 2 (D4). Supporting employee removed everywhere (0 of 185 stored tasks used it). The drawer names who asked and who approves and when; team tasks say who they went to (fewest open tasks). Helpers hear status changes and overdue reminders.</t>
+        </is>
+      </c>
+      <c r="G189" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H189" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I189" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J189" s="28" t="n"/>
+      <c r="K189" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 93686c2 + tracker c365e38 (2026-09-14). 3 real-save journeys; browser check writes blocked.</t>
+        </is>
+      </c>
+      <c r="L189" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.9</t>
+        </is>
+      </c>
+      <c r="B190" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, services/tasks.py + counts</t>
+        </is>
+      </c>
+      <c r="C190" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D190" s="28" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E190" s="28" t="inlineStr">
+        <is>
+          <t>Stages and flags -- To do / Doing / Done, Waiting on someone</t>
+        </is>
+      </c>
+      <c r="F190" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-07 / plan Phase 3 (D6). Screens show three stages; stored statuses unchanged (no migration). Waiting on a colleague or a typed name, with since when; the colleague is told and can answer with a note. Status filter To do / Doing / Waiting on someone / Needs approval / Overdue / Due today / Done. Operating Score, calendar, dashboard, Brief, prioritisation and leave impact count waiting and review as open work.</t>
+        </is>
+      </c>
+      <c r="G190" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H190" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I190" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J190" s="28" t="n"/>
+      <c r="K190" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED abe4b40 (2026-09-14). 10 unit tests, 2 real-save journeys, browser 13/13. Dex counts handed to Yokesh (agent_tools.py, brain.py), not changed here.</t>
+        </is>
+      </c>
+      <c r="L190" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.10</t>
+        </is>
+      </c>
+      <c r="B191" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, lib/taskAccess.js, routers/tasks.py</t>
+        </is>
+      </c>
+      <c r="C191" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D191" s="28" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="E191" s="28" t="inlineStr">
+        <is>
+          <t>Task access -- who may assign, who sees all tasks</t>
+        </is>
+      </c>
+      <c r="F191" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 TK-08 / plan 6.1-6.6 (D1). New permissions Assign tasks to anyone and See all tasks, off for every role (finance included). Without the first, work goes to yourself, your team or your reports -- on create, change and reassign, and the pickers list only those. All Tasks for the owner and See all tasks holders. Creating needs the Tasks permission. /auth/me sends effective_permissions.</t>
+        </is>
+      </c>
+      <c r="G191" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H191" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I191" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J191" s="28" t="n"/>
+      <c r="K191" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED b2ae273 (2026-09-14). Browser 49/49 across 4 roles desktop + phone; 7 unit tests; real-save journeys for every refusal.</t>
+        </is>
+      </c>
+      <c r="L191" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.11</t>
+        </is>
+      </c>
+      <c r="B192" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js, lib/taskAccess.js, routers/tasks.py</t>
+        </is>
+      </c>
+      <c r="C192" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D192" s="28" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="E192" s="28" t="inlineStr">
+        <is>
+          <t>Who may change a task -- the people who run it, not the whole company</t>
+        </is>
+      </c>
+      <c r="F192" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 item 7 / plan 6.7. PATCH /tasks/{id} was open to any member. Now: stage / progress / waiting -- doer, helpers, asker, manager, owner; done / cancel / reopen -- the same minus helpers; people -- asker, manager, Manage Team, owner; priority -- asker, manager, owner; needs proof -- asker and owner. See all tasks, the approver and a colleague waited on leave notes. Drawer and bulk Complete / Reassign follow it.</t>
+        </is>
+      </c>
+      <c r="G192" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H192" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I192" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J192" s="28" t="n"/>
+      <c r="K192" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 92c3d0f (2026-09-15). Browser 96/96 per relationship desktop + phone; 6 unit tests; real-save journey test_who_may_change_a_task.</t>
+        </is>
+      </c>
+      <c r="L192" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.12</t>
+        </is>
+      </c>
+      <c r="B193" s="28" t="inlineStr">
+        <is>
+          <t>finance_signals.py, routers/desk.py, MyWork.js</t>
+        </is>
+      </c>
+      <c r="C193" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D193" s="28" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="E193" s="28" t="inlineStr">
+        <is>
+          <t>Stuck work reaches the manager first -- reminders, Escalate, Desk Slipping</t>
+        </is>
+      </c>
+      <c r="F193" s="28" t="inlineStr">
+        <is>
+          <t>ASK-28 plan Phase 7 (D7). Overdue: the people who can move it (the approver for approval, the colleague waited on); 1 day: again; 2 days: the doer's reporting manager (the owner only without one); 4 days: owner alert (was 3). Escalate goes to your manager first. Desk Slipping shows a manager their reports' work from 2 days, and now shows escalations at all (it read the wrong field names).</t>
+        </is>
+      </c>
+      <c r="G193" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H193" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I193" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J193" s="28" t="n"/>
+      <c r="K193" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 92c3d0f (2026-09-15). 4 unit tests + ladder test updated; real-save journey test_stuck_work_reaches_the_right_person; Escalate browser 15/15; Desk probe 4/4 read-only on real data. Goes live when the backend is restarted or deployed.</t>
+        </is>
+      </c>
+      <c r="L193" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.13</t>
+        </is>
+      </c>
+      <c r="B194" s="28" t="inlineStr">
+        <is>
+          <t>backend/tests, backend/scripts</t>
+        </is>
+      </c>
+      <c r="C194" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D194" s="28" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="E194" s="28" t="inlineStr">
+        <is>
+          <t>Safe testing -- real saves in an isolated database, browser checks with writes blocked</t>
+        </is>
+      </c>
+      <c r="F194" s="28" t="inlineStr">
+        <is>
+          <t>The local database is production, so every browser acceptance script aborts POST/PATCH/PUT/DELETE after sign-in, and real saves run in tests/test_task_management_e2e.py against a throwaway with_test_db. The two old My Work audit scripts that created real tasks now refuse to run without UX_ALLOW_WRITES=1.</t>
+        </is>
+      </c>
+      <c r="G194" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H194" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I194" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J194" s="28" t="n"/>
+      <c r="K194" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 009bd2d and with each phase (2026-09-14/15). Full suite 1452 passed at 92c3d0f.</t>
+        </is>
+      </c>
+      <c r="L194" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.14</t>
+        </is>
+      </c>
+      <c r="B195" s="28" t="inlineStr">
+        <is>
+          <t>mobile/ (Flutter)</t>
+        </is>
+      </c>
+      <c r="C195" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D195" s="28" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E195" s="28" t="inlineStr">
+        <is>
+          <t>Flutter app catches up with the task changes</t>
+        </is>
+      </c>
+      <c r="F195" s="28" t="inlineStr">
+        <is>
+          <t>The Flutter app still shows stored status words (not To do / Doing / Done), still offers Complete to helpers (the server refuses with the reason), and its Escalate does not say it goes to the manager. It keeps working because nothing stored changed.</t>
+        </is>
+      </c>
+      <c r="G195" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H195" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I195" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J195" s="28" t="n"/>
+      <c r="K195" s="28" t="inlineStr">
+        <is>
+          <t>Open follow-up from the task management plan (plan 0.5).</t>
+        </is>
+      </c>
+      <c r="L195" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.15</t>
+        </is>
+      </c>
+      <c r="B196" s="28" t="inlineStr">
+        <is>
+          <t>backend/.env, test setup</t>
+        </is>
+      </c>
+      <c r="C196" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D196" s="28" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="E196" s="28" t="inlineStr">
+        <is>
+          <t>Separate the local database from production</t>
+        </is>
+      </c>
+      <c r="F196" s="28" t="inlineStr">
+        <is>
+          <t>Local MONGO_URL points at production, so real-click testing is impossible and the local backend cannot be restarted with new reminder rules without messaging real people. A separate test database unblocks both.</t>
+        </is>
+      </c>
+      <c r="G196" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H196" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I196" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J196" s="28" t="n"/>
+      <c r="K196" s="28" t="inlineStr">
+        <is>
+          <t>Open follow-up from the task management plan (plan 0.1).</t>
+        </is>
+      </c>
+      <c r="L196" s="28" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-09-14 (docs/TASK_MANAGEMENT_PLAN.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Proof stays once the work is completed; API baseline for attachment removal
- Nobody, the owner included, removes proof from a task that is done or
  sent for sign-off; reopen it to change the proof. Reference material
  stays removable. My Work hides the remove button in the same cases.
- Real-save journey test_proof_stays_once_the_work_is_completed.
- API parity baseline regenerated for DELETE /tasks/{id}/attachments/{att_id}
  (added in bb0a9e8).
- Decision Desk plan: 3.5 sign-off before done on decision tasks (another
  team); automatic proof on Finance tasks not needed. Trackers updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -2299,14 +2299,14 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D26" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Task management plan (docs/TASK_MANAGEMENT_PLAN.md), ASK-28 + ASK-29, 2026-09-14/15: New Task form, Asked by me / Waiting for my approval / My team views, links that land, approval moment, who is on a task, stages and flags, task access, who may change a task, stuck work reaches the manager first. Open: Flutter app, separate test database.</t>
+          <t>Task management plan (docs/TASK_MANAGEMENT_PLAN.md), ASK-28 + ASK-29, 2026-09-14/15: New Task form, Asked by me / Waiting for my approval / My team views, links that land, approval moment, who is on a task, stages and flags, task access, who may change a task, stuck work reaches the manager first, proof stays once work is completed. Open: Flutter app, separate test database.</t>
         </is>
       </c>
     </row>
@@ -2335,11 +2335,11 @@
         <v>12</v>
       </c>
       <c r="D27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves. Open: Phase 5 (capture feedback on desktop, retry, My captures).</t>
+          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves. Open: sign-off before done on decision tasks (3.5, another team), Phase 5 (capture feedback on desktop, retry, My captures).</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>(this push)</t>
+          <t>9dcb046</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>(this push)</t>
+          <t>9dcb046</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
@@ -5501,20 +5501,47 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
+          <t>9dcb046</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>ASK-32 Phases 3-4 - simple decision screen with edits; workflows matched and moved by themselves</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
           <t>(this push)</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
+      <c r="C120" s="7" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t>ASK-32 Phases 3-4 - simple decision screen with edits; workflows matched and moved by themselves</t>
-        </is>
-      </c>
-      <c r="E119" s="7" t="inlineStr">
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>Proof stays once the work is completed (done or sent for sign-off); reopen to change it</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -5531,7 +5558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L209"/>
+  <dimension ref="A1:L211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17354,6 +17381,118 @@
         </is>
       </c>
       <c r="L209" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="28" t="inlineStr">
+        <is>
+          <t>U7-21.16</t>
+        </is>
+      </c>
+      <c r="B210" s="28" t="inlineStr">
+        <is>
+          <t>routers/tasks.py, MyWork.js</t>
+        </is>
+      </c>
+      <c r="C210" s="28" t="n">
+        <v>21</v>
+      </c>
+      <c r="D210" s="28" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="E210" s="28" t="inlineStr">
+        <is>
+          <t>Proof stays once the work is completed</t>
+        </is>
+      </c>
+      <c r="F210" s="28" t="inlineStr">
+        <is>
+          <t>Removing an attachment (DELETE /tasks/{id}/attachments/{att_id}, added in bb0a9e8) let the uploader, the creator or the owner remove proof at any time, so a closed task could lose its evidence. Now nobody, the owner included, removes proof while the task is done or sent for sign-off; reopen the task to change it. Reference material stays removable. My Work hides the remove button in the same cases.</t>
+        </is>
+      </c>
+      <c r="G210" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H210" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I210" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J210" s="28" t="n"/>
+      <c r="K210" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED (this push, 2026-09-15). Real-save journey test_proof_stays_once_the_work_is_completed (open, sent for sign-off, done, reopened).</t>
+        </is>
+      </c>
+      <c r="L210" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="28" t="inlineStr">
+        <is>
+          <t>U7-22.14</t>
+        </is>
+      </c>
+      <c r="B211" s="28" t="inlineStr">
+        <is>
+          <t>DecisionDialog.js, services/decision_flow.py, services/voice.py</t>
+        </is>
+      </c>
+      <c r="C211" s="28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D211" s="28" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="E211" s="28" t="inlineStr">
+        <is>
+          <t>Needs sign-off before done on decision tasks</t>
+        </is>
+      </c>
+      <c r="F211" s="28" t="inlineStr">
+        <is>
+          <t>Plan 3.5. One checkbox per task row on the decision screen (only for whoever decides). On approval the task needs sign-off before it closes, and the decision's approver signs off. Dex ticks it in advance for Finance tasks or amounts at or above the high-value threshold. No approval before start.</t>
+        </is>
+      </c>
+      <c r="G211" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H211" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I211" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J211" s="28" t="n"/>
+      <c r="K211" s="28" t="inlineStr">
+        <is>
+          <t>Planned in docs/DECISION_DESK_PLAN.md 3.5. Being built by another team (Yokesh 2026-09-15).</t>
+        </is>
+      </c>
+      <c r="L211" s="28" t="inlineStr">
         <is>
           <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
         </is>

</xml_diff>

<commit_message>
Needs approval is task approvals only; decision card says who raised it and who decides
- My Work's Needs approval filter lists task approvals only (before start,
  sent back, sign-off). Tasks waiting for a decision stay in All tasks with
  their decision link; decisions are approved on the Desk.
- Desk decision card: "Raised by Priya · You decide · Waiting 13 days ·
  Unblocks 2 tasks", or "Raised by you · Sunita decides" when following.
- scripts/cleanup_test_data_0915.py: archives, then removes old test tasks
  and decisions with nothing to act on; --restore puts a run back.
- Decision Desk plan: tidy-up section, DD5/DD6 ticked, Phase 5 later.
  Trackers updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -2332,14 +2332,14 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D27" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves. Open: sign-off before done on decision tasks (3.5, another team), Phase 5 (capture feedback on desktop, retry, My captures).</t>
+          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves; Needs approval is task approvals only; the card says who raised it and who decides; test data cleared. Open: sign-off before done on decision tasks (3.5, another team), Phase 5 (capture feedback on desktop, retry, My captures).</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E120"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5528,20 +5528,47 @@
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
+          <t>5dad142</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>Proof stays once the work is completed (done or sent for sign-off); reopen to change it</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>Decision Desk decision flow</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
           <t>(this push)</t>
         </is>
       </c>
-      <c r="C120" s="7" t="inlineStr">
+      <c r="C121" s="7" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D120" s="7" t="inlineStr">
-        <is>
-          <t>Proof stays once the work is completed (done or sent for sign-off); reopen to change it</t>
-        </is>
-      </c>
-      <c r="E120" s="7" t="inlineStr">
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Needs approval is task approvals only; decision card says who raised it and who decides</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -5558,7 +5585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L211"/>
+  <dimension ref="A1:L214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17493,6 +17520,174 @@
         </is>
       </c>
       <c r="L211" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="28" t="inlineStr">
+        <is>
+          <t>U7-22.15</t>
+        </is>
+      </c>
+      <c r="B212" s="28" t="inlineStr">
+        <is>
+          <t>MyWork.js</t>
+        </is>
+      </c>
+      <c r="C212" s="28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D212" s="28" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="E212" s="28" t="inlineStr">
+        <is>
+          <t>Needs approval is task approvals only</t>
+        </is>
+      </c>
+      <c r="F212" s="28" t="inlineStr">
+        <is>
+          <t>My Work's Needs approval filter counted every blocked task, so 32 tasks waiting for a decision sat beside the 7 task approvals (39). Decisions are approved on the Desk only; the filter now lists task approvals (before start, sent back, sign-off). Decision-locked tasks stay in All tasks with Waiting for a decision and a link.</t>
+        </is>
+      </c>
+      <c r="G212" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H212" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I212" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J212" s="28" t="n"/>
+      <c r="K212" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED (this push, 2026-09-15).</t>
+        </is>
+      </c>
+      <c r="L212" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="28" t="inlineStr">
+        <is>
+          <t>U7-22.16</t>
+        </is>
+      </c>
+      <c r="B213" s="28" t="inlineStr">
+        <is>
+          <t>routers/desk.py</t>
+        </is>
+      </c>
+      <c r="C213" s="28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D213" s="28" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="E213" s="28" t="inlineStr">
+        <is>
+          <t>Decision card says who raised it and who decides</t>
+        </is>
+      </c>
+      <c r="F213" s="28" t="inlineStr">
+        <is>
+          <t>Desk decision card: Raised by Priya · You decide · Waiting 13 days · Unblocks 2 tasks; the person following it sees Raised by you · Sunita decides.</t>
+        </is>
+      </c>
+      <c r="G213" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H213" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I213" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J213" s="28" t="n"/>
+      <c r="K213" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED (this push, 2026-09-15). test_decision_flow_e2e asserts both lines.</t>
+        </is>
+      </c>
+      <c r="L213" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="28" t="inlineStr">
+        <is>
+          <t>U7-22.17</t>
+        </is>
+      </c>
+      <c r="B214" s="28" t="inlineStr">
+        <is>
+          <t>scripts/cleanup_test_data_0915.py</t>
+        </is>
+      </c>
+      <c r="C214" s="28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D214" s="28" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="E214" s="28" t="inlineStr">
+        <is>
+          <t>Old test tasks and empty decisions cleared</t>
+        </is>
+      </c>
+      <c r="F214" s="28" t="inlineStr">
+        <is>
+          <t>Sharma company (dev data): 60 test tasks, 22 decisions with nothing to act on, and their 62 notifications and 113 activity entries. Archived to cleanup_archive first; --restore puts a run back.</t>
+        </is>
+      </c>
+      <c r="G214" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H214" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I214" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J214" s="28" t="n"/>
+      <c r="K214" s="28" t="inlineStr">
+        <is>
+          <t>DONE (2026-09-15).</t>
+        </is>
+      </c>
+      <c r="L214" s="28" t="inlineStr">
         <is>
           <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
         </is>

</xml_diff>

<commit_message>
Every approval task names who approves; Settings / Team / RBAC review
- A task that needs approval with nobody picked: the creator's reporting
  manager when they may approve tasks, else the owner (an owner approves
  their own; with several owners, the first). A picked approver wins.
  New Task shows the default instead of "Anyone with approval access", so
  My approvals covers every task and only that person is told.
- Real-save journey test_nobody_picked_the_manager_approves_else_the_owner;
  live test iteration47 updated to the rule.
- docs/SETTINGS_RBAC_REVIEW.md: section-by-section review of Settings, Team,
  roles/permissions, task and decision access, with P0/P1/P2 findings.
- Decision Desk plan and trackers updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -2332,14 +2332,14 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves; Needs approval is task approvals only; the card says who raised it and who decides; test data cleared. Open: sign-off before done on decision tasks (3.5, another team), Phase 5 (capture feedback on desktop, retry, My captures).</t>
+          <t>Decision Desk decision flow (docs/DECISION_DESK_PLAN.md), ASK-32, 2026-09-15: proposals until approval, who decides and who is told, a simple editable decision screen, workflows matched and moved by themselves; Needs approval is task approvals only; the card says who raised it and who decides; test data cleared; every approval task names who approves (manager, else owner). Open: sign-off before done on decision tasks (3.5, another team), Phase 5 (capture feedback on desktop, retry, My captures).</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5555,20 +5555,47 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
+          <t>963e7d3</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Needs approval is task approvals only; decision card says who raised it and who decides</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>My Work task management</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
           <t>(this push)</t>
         </is>
       </c>
-      <c r="C121" s="7" t="inlineStr">
+      <c r="C122" s="7" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D121" s="7" t="inlineStr">
-        <is>
-          <t>Needs approval is task approvals only; decision card says who raised it and who decides</t>
-        </is>
-      </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>Every approval task names who approves: the creator's manager, else the owner</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -5585,7 +5612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L214"/>
+  <dimension ref="A1:L215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17688,6 +17715,62 @@
         </is>
       </c>
       <c r="L214" s="28" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="28" t="inlineStr">
+        <is>
+          <t>U7-22.18</t>
+        </is>
+      </c>
+      <c r="B215" s="28" t="inlineStr">
+        <is>
+          <t>routers/tasks.py, Tasks.js</t>
+        </is>
+      </c>
+      <c r="C215" s="28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D215" s="28" t="inlineStr">
+        <is>
+          <t>Approval</t>
+        </is>
+      </c>
+      <c r="E215" s="28" t="inlineStr">
+        <is>
+          <t>Every approval task names who approves</t>
+        </is>
+      </c>
+      <c r="F215" s="28" t="inlineStr">
+        <is>
+          <t>Needs approval with nobody picked: the creator's reporting manager when they may approve tasks, else the owner (an owner creating it approves it; with several owners the first). A picked approver wins. New Task shows the default in the Approver list instead of Anyone with approval access, so My approvals covers every task and only that person is told.</t>
+        </is>
+      </c>
+      <c r="G215" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H215" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I215" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J215" s="28" t="n"/>
+      <c r="K215" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED (this push, 2026-09-15). Real-save journey test_nobody_picked_the_manager_approves_else_the_owner.</t>
+        </is>
+      </c>
+      <c r="L215" s="28" t="inlineStr">
         <is>
           <t>Yokesh 2026-09-15 (docs/DECISION_DESK_PLAN.md)</t>
         </is>

</xml_diff>

<commit_message>
Settings opens again for everyone but an owner
ASK-33 Phase 5 (2eed722) took the theme switch out — the app is light-only now
— and dropped the Appearance card from the owner's Account tab, but the
non-owner view still rendered <ThemeCard />. So Settings threw "ThemeCard is
not defined" for every teammate: the broken-panel notice instead of the page,
with language, profile, password, hand-over and sign out all out of reach.

Caught by the RBAC browser checks after rebasing onto it. The P2 check now
looks for what the page actually holds (language and hand-over, no Appearance
card) rather than what it held yesterday.

Verified: browser acceptance on a throwaway database, P1 23/23 and P2 32/32.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -2365,14 +2365,14 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D28" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2397,7 +2397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5769,6 +5769,33 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>Settings, Team and access</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t>(this push)</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t>Settings opens again for everyone but an owner (the Appearance card was removed from one branch only)</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5780,7 +5807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L241"/>
+  <dimension ref="A1:L242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19397,6 +19424,62 @@
       <c r="L241" s="28" t="inlineStr">
         <is>
           <t>Found re-checking the Team page after 8b60707</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.27</t>
+        </is>
+      </c>
+      <c r="B242" s="28" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Settings.js</t>
+        </is>
+      </c>
+      <c r="C242" s="28" t="n">
+        <v>23</v>
+      </c>
+      <c r="D242" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E242" s="28" t="inlineStr">
+        <is>
+          <t>Settings opened again for everyone but an owner</t>
+        </is>
+      </c>
+      <c r="F242" s="28" t="inlineStr">
+        <is>
+          <t>ASK-33 Phase 5 (2eed722) dropped the Appearance card with the theme switch, but the non-owner view still rendered &lt;ThemeCard /&gt;: the page threw "ThemeCard is not defined" and every teammate got the broken-panel notice instead of Settings — language, profile, password, hand-over and sign out all unreachable.</t>
+        </is>
+      </c>
+      <c r="G242" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H242" s="28" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I242" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J242" s="28" t="n"/>
+      <c r="K242" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED (this push, 2026-09-16). Caught by the P1/P2 browser checks after rebasing onto 2eed722; browser ux_rbac_p1_0916.py 23/23 and ux_rbac_p2_0916.py 32/32 on a throwaway database.</t>
+        </is>
+      </c>
+      <c r="L242" s="28" t="inlineStr">
+        <is>
+          <t>Found re-running the RBAC browser checks</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Chinmay's two commits get their rows
Neither 53f76ab (CRM three kinds, delete and resolve) nor 10111ee (Later is
Save as draft) carried a tracker row, so the sheet did not say the work had
happened.

- U7-25.33: the CRM's three kinds, each with its own door, plus delete and
  resolve; notes that no tests came with it and that the browser check after
  it (U7-25.32) found five unfinished things, now fixed.
- U7-25.34: "Save as draft" and the draft mark; notes the mark is per-device
  (localStorage) and that docs/PILOT-2_DRAFT_FLAG_ASK.md is still an open ask.

Sprint 25 26/34, epic 215/318.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 213 of 316 items Done  (67%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 31 of 32 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 24 of 32 Done.</t>
+          <t>Epic 6 progress: 215 of 318 items Done  (67%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 31 of 32 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 26 of 34 Done.</t>
         </is>
       </c>
     </row>
@@ -2431,14 +2431,14 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D30" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -6035,7 +6035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L317"/>
+  <dimension ref="A1:L319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23864,6 +23864,120 @@
       <c r="L317" s="28" t="inlineStr">
         <is>
           <t>Yokesh 2026-09-27 (browser check of J15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.33</t>
+        </is>
+      </c>
+      <c r="B318" s="28" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/CRM.js, pages/ContactProfile.js (Chinmay, commit 53f76ab)</t>
+        </is>
+      </c>
+      <c r="C318" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D318" s="28" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="E318" s="28" t="inlineStr">
+        <is>
+          <t>Three kinds, each with its own door — customers, partners and suppliers, plus delete and resolve</t>
+        </is>
+      </c>
+      <c r="F318" s="28" t="inlineStr">
+        <is>
+          <t>Six things the founder found, all the same shape: the CRM knew how to do something and gave nobody a way to ask for it. A dealer could only be made by adding a customer and flipping the type inside the window, and that flip stayed live on every later edit — a contact could change sides with one tap. Partners were folded into the customers list with no way to see them. A contact added by mistake stayed for ever (DELETE /contacts/:id existed, nothing called it). A complaint could be logged and then closed from nowhere (PATCH /complaints/:id/resolve existed, nothing called it), so the red count only climbed.</t>
+        </is>
+      </c>
+      <c r="G318" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H318" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I318" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K318" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-09-26 by Chinmay (53f76ab), frontend only — every endpoint it needed already existed. Each kind has its own entry in Add contact, its own tab, and no way to change what a contact is after it exists (wrong kind = delete and add again). Partners get a tab under that name; both are the buyer side, so they open and close together with crm_buyers and nobody gains access by the split. Deleting the contact a profile page is ABOUT leaves that page. Verified on the running stack by the author. NOT in that commit: tests, and tracker rows — this row is the record; the browser check afterwards (U7-25.32) found five things it had not finished, all now fixed.</t>
+        </is>
+      </c>
+      <c r="L318" s="28" t="inlineStr">
+        <is>
+          <t>Chinmay 2026-09-26 (founder's six CRM findings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.34</t>
+        </is>
+      </c>
+      <c r="B319" s="28" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/desk/DeskDexWell.jsx, pages/Desk.js, components/DecisionDialog.js, lib/deferredDecisions.js (Chinmay, commit 10111ee)</t>
+        </is>
+      </c>
+      <c r="C319" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D319" s="28" t="inlineStr">
+        <is>
+          <t>Decision Desk</t>
+        </is>
+      </c>
+      <c r="E319" s="28" t="inlineStr">
+        <is>
+          <t>"Later" is "Save as draft", and a draft says so</t>
+        </is>
+      </c>
+      <c r="F319" s="28" t="inlineStr">
+        <is>
+          <t>The pilot client's second voice note: the button after Dex reads a capture should say Save as draft, and the tinted row in the Decisions column should carry the word, not the colour alone.</t>
+        </is>
+      </c>
+      <c r="G319" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H319" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I319" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K319" s="28" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-09-27 by Chinmay (10111ee). The well's ending offers 'Save as draft' where it said 'Later' (testid desk-dex-later kept, so the suites still find it); the Desk's Decisions row says 'Draft' in its meta line instead of 'Set aside'; DecisionDialog carries '(Draft)' after the title wherever it opens while the decision can still be decided; a draft stays a draft until it is decided — opening it no longer clears the mark, approving or rejecting does. OPEN: the mark is per-device (localStorage) — the decision is on the server, the draft flag is not, so it does not follow the founder to their phone. docs/PILOT-2_DRAFT_FLAG_ASK.md is the backend ask that would make it travel; not yet built. No tests in the commit.</t>
+        </is>
+      </c>
+      <c r="L319" s="28" t="inlineStr">
+        <is>
+          <t>Pilot client via Chinmay 2026-09-27 (PILOT-2 B)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor ones: reset link checked up front, admin console restyled and fast
- A dead reset link now says so before the form: new read-only
  POST /auth/password/reset/check (auth_emails.is_live) previews consume()
  without spending the token. CSRF-exempt, public allow-list, API baseline +1.
- <option> elements hold one string (admin Support/Config, Tasks picker):
  the only console error across all 17 admin tabs.
- The admin console is drawn in the app's own style via one shared
  adminStyle.js; status colours darkened for a light ground. All 17 tabs
  measured at >= 4.5:1 contrast, no overflow at 390px, testids kept.
- GET /admin/tenants asked 4 queries per workspace in series (24 s for 13);
  now 4 grouped queries in parallel (0.8 s), response byte-identical.
  Support ticket counts asked together.

Tracker: U7-25.85-88 (Sprint 25 80/88, Epic 6 273/371).
Full suite: 1987 passed, 645 skipped, 0 failed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 269 of 367 items Done  (73%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 31 of 32 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 76 of 84 Done.</t>
+          <t>Epic 6 progress: 273 of 371 items Done  (74%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 31 of 32 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2436,17 +2436,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>80</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -6043,7 +6043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L369"/>
+  <dimension ref="A1:L373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26859,6 +26859,234 @@
       <c r="L369" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-03 (full-product pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.85</t>
+        </is>
+      </c>
+      <c r="B370" s="28" t="inlineStr">
+        <is>
+          <t>frontend pages/PasswordReset.js + backend /auth/password/reset/check</t>
+        </is>
+      </c>
+      <c r="C370" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D370" s="28" t="inlineStr">
+        <is>
+          <t>Error states</t>
+        </is>
+      </c>
+      <c r="E370" s="28" t="inlineStr">
+        <is>
+          <t>A dead reset link says so before the form, not after</t>
+        </is>
+      </c>
+      <c r="F370" s="28" t="inlineStr">
+        <is>
+          <t>A spent or expired reset link showed 'Set a new password', let the founder choose one and type it twice, and only then said the link was dead.</t>
+        </is>
+      </c>
+      <c r="G370" s="28" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H370" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I370" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. New POST /auth/password/reset/check (auth_emails.is_live) previews consume() without spending the token; the page shows 'Checking your link…' then either the form or 'This link won't work'. If the check cannot be asked, the form shows and the reset decides. CSRF-exempt like reset; API baseline regenerated (+1 route). Verified: live token shows the form and stays unspent; dead token goes straight to the dead state.</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (minor ones from the full-product pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.86</t>
+        </is>
+      </c>
+      <c r="B371" s="28" t="inlineStr">
+        <is>
+          <t>frontend admin Support/Config + pages/Tasks.js</t>
+        </is>
+      </c>
+      <c r="C371" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D371" s="28" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="E371" s="28" t="inlineStr">
+        <is>
+          <t>An &lt;option&gt; holds one string</t>
+        </is>
+      </c>
+      <c r="F371" s="28" t="inlineStr">
+        <is>
+          <t>Text plus expressions inside &lt;option&gt; rendered invalid markup in development -- the only console error across all 17 admin console tabs.</t>
+        </is>
+      </c>
+      <c r="G371" s="28" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H371" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I371" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. Support status filter, Config's default-model option and the Tasks assignee picker each render one template string. Verified: zero console errors across all 17 admin tabs.</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (minor ones from the full-product pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.87</t>
+        </is>
+      </c>
+      <c r="B372" s="28" t="inlineStr">
+        <is>
+          <t>frontend pages/admin/* (12 files) + adminStyle.js</t>
+        </is>
+      </c>
+      <c r="C372" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D372" s="28" t="inlineStr">
+        <is>
+          <t>Visual consistency</t>
+        </is>
+      </c>
+      <c r="E372" s="28" t="inlineStr">
+        <is>
+          <t>The admin console is drawn in the app's own style</t>
+        </is>
+      </c>
+      <c r="F372" s="28" t="inlineStr">
+        <is>
+          <t>The platform console was the last surface in the retired brutalist dark style: black ground, mono uppercase buttons, square borders, and six style constants copied into every section.</t>
+        </is>
+      </c>
+      <c r="G372" s="28" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H372" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I372" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. One shared adminStyle.js (glass cards, pills, quiet labels from components/karma/glass); every section imports it. Shell and login rewritten by hand; the red stays as the console's mark so it is never mistaken for a tenant screen. Measured in the browser: every text element on all 17 tabs passes 4.5:1 contrast (status colours darkened for a light ground), no horizontal overflow at 390px, zero console errors. All data-testids kept.</t>
+        </is>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (minor ones from the full-product pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="28" t="inlineStr">
+        <is>
+          <t>U7-25.88</t>
+        </is>
+      </c>
+      <c r="B373" s="28" t="inlineStr">
+        <is>
+          <t>backend routers/admin.py GET /admin/tenants (+ admin_support counts)</t>
+        </is>
+      </c>
+      <c r="C373" s="28" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D373" s="28" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="E373" s="28" t="inlineStr">
+        <is>
+          <t>The workspace list loads in under a second instead of 24</t>
+        </is>
+      </c>
+      <c r="F373" s="28" t="inlineStr">
+        <is>
+          <t>Found while checking the restyle: Workspaces sat on Loading… -- the endpoint asked four questions PER workspace in sequence (52 round trips for 13 workspaces), 24 s against the hosted database and growing with every customer.</t>
+        </is>
+      </c>
+      <c r="G373" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H373" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I373" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. Four grouped aggregations for all workspaces, run concurrently: 24 s -&gt; 0.8 s warm, response byte-identical to the old one (compared in the browser). Support ticket status counts also asked together instead of in series.</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (minor ones from the full-product pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A file follows its record
/files/{id}/download served any file to any member holding its id. Now
routers/files.may_read_file asks the record's question: profile photos to the
company; your own uploads; a task's attachment to whoever may open the task
(may_read_task, extracted from get_task so both share it); a capture's or
decision's reference to whoever may open that note or decision; the owner
everything. The legacy /files/{name} route asks the same, plus Finance or Data
Input for uploaded bills, Finance for ledger attachments, and the review queue
for AI-draft previews.

Verified on the scratch company: a photo on the sales member's task opened
for her and the owner and was refused (403) to the finance member, on both
routes.

Tests: test_a_file_follows_its_record. Tracker: U7-23.40 Done (Sprint 23 46/47).
Full suite: 2057 passed, 645 skipped, 0 failed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 287 of 386 items Done  (74%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 45 of 47 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
+          <t>Epic 6 progress: 288 of 386 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 46 of 47 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -27593,12 +27593,12 @@
       </c>
       <c r="I382" s="28" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>Not changed: a record-aware check needs each file to know its owning record and kind -- a contained follow-up.</t>
+          <t>SHIPPED 2026-10-03 (founder). routers/files.may_read_file: avatars to the company; your own uploads; a task's attachment to whoever may open the task (may_read_task, extracted from get_task); a capture's or decision's reference to whoever may open that note or decision; the owner everything. The legacy /files/{name} route asks the same, plus Finance/Data Input for uploaded bills, Finance for ledger attachments and the review queue for AI-draft previews. Verified: a photo on Priya's task opened for her and the owner, 403 for Anand, on both routes.</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">

</xml_diff>

<commit_message>
Settings and the desktop say only what applies
Settings (walked as owner, default member and finance member):
- The audit log names people; mobile sign-ins read "A member" before.
- "AI keys" named its WhatsApp rows (were Wa_access_token /
  Wa_phone_number_id) and is titled "AI and WhatsApp keys".
- Leave approvers no longer point at the retired "People -> Employees".
- "While you're away" shows only to people with approvals to hand over.

Desktop:
- Finance has no "Photo" button on desktop (it opened the same picker as
  "Upload bill / receipt"); the phone keeps it.
- The install-the-app bar is phone-only.

Gaps recorded as Backlog: upgrade/pay path (checkout exists, no UI), active
sessions + sign out everywhere, notification preferences, owner data export,
Teams & access as its own tab.

Tests: test_settings_and_desktop_say_only_what_applies. Tracker: U7-23.47-55.
Full suite: 2063 passed, 645 skipped, 0 failed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 288 of 386 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 46 of 47 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
+          <t>Epic 6 progress: 292 of 395 items Done  (74%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 50 of 56 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2370,17 +2370,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L388"/>
+  <dimension ref="A1:L397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27946,6 +27946,519 @@
       <c r="L388" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-03 (role system product review, browser end to end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.47</t>
+        </is>
+      </c>
+      <c r="B389" s="28" t="inlineStr">
+        <is>
+          <t>routers/tenant_settings.py read_audit_log; Settings.js</t>
+        </is>
+      </c>
+      <c r="C389" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D389" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E389" s="28" t="inlineStr">
+        <is>
+          <t>The audit log names people</t>
+        </is>
+      </c>
+      <c r="F389" s="28" t="inlineStr">
+        <is>
+          <t>Every member who signs in by mobile has no email, so the owner's audit log read 'Logout — A member' for all of them.</t>
+        </is>
+      </c>
+      <c r="G389" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H389" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I389" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. The endpoint resolves actor ids to names; the table shows name, else email. Verified: Priya Nair, Anand Rao, Kavya Raman.</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.48</t>
+        </is>
+      </c>
+      <c r="B390" s="28" t="inlineStr">
+        <is>
+          <t>Settings.js AiKeysCard; Leave.js</t>
+        </is>
+      </c>
+      <c r="C390" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D390" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E390" s="28" t="inlineStr">
+        <is>
+          <t>Keys and approvers described in words</t>
+        </is>
+      </c>
+      <c r="F390" s="28" t="inlineStr">
+        <is>
+          <t>'AI keys' listed Wa_access_token and Wa_phone_number_id as if they were AI providers; Leave approvers pointed at 'People → Employees', retired.</t>
+        </is>
+      </c>
+      <c r="G390" s="28" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H390" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I390" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. WhatsApp rows named; card titled 'AI and WhatsApp keys'; leave copy points at the Team card.</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.49</t>
+        </is>
+      </c>
+      <c r="B391" s="28" t="inlineStr">
+        <is>
+          <t>Settings.js DelegationCard</t>
+        </is>
+      </c>
+      <c r="C391" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D391" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E391" s="28" t="inlineStr">
+        <is>
+          <t>The hand-over is offered only to people with approvals</t>
+        </is>
+      </c>
+      <c r="F391" s="28" t="inlineStr">
+        <is>
+          <t>'While you're away — hand your approvals' showed to a member who approves nothing.</t>
+        </is>
+      </c>
+      <c r="G391" s="28" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H391" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I391" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. Shows for the owner, approval-permission holders, anyone with direct reports, or a hand-over already running. Verified: Priya no card, Anand card.</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.50</t>
+        </is>
+      </c>
+      <c r="B392" s="28" t="inlineStr">
+        <is>
+          <t>Ledger.js; mobile/InstallPrompt.jsx</t>
+        </is>
+      </c>
+      <c r="C392" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D392" s="28" t="inlineStr">
+        <is>
+          <t>Desktop</t>
+        </is>
+      </c>
+      <c r="E392" s="28" t="inlineStr">
+        <is>
+          <t>Desktop shows only what a desktop can use</t>
+        </is>
+      </c>
+      <c r="F392" s="28" t="inlineStr">
+        <is>
+          <t>Finance on desktop offered 'Photo', which opened the same file picker as 'Upload bill / receipt'; desktop Chrome was offered the phone app's install bar.</t>
+        </is>
+      </c>
+      <c r="G392" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H392" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I392" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-03. Photo kept on the phone only; install bar phone-only. Swept 14 desktop pages for phone-only wording or camera buttons: none left.</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.51</t>
+        </is>
+      </c>
+      <c r="B393" s="28" t="inlineStr">
+        <is>
+          <t>Settings &gt; Workspace &gt; Plan and seats; routers/billing.py</t>
+        </is>
+      </c>
+      <c r="C393" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D393" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E393" s="28" t="inlineStr">
+        <is>
+          <t>An owner can pay: Upgrade / Choose plan</t>
+        </is>
+      </c>
+      <c r="F393" s="28" t="inlineStr">
+        <is>
+          <t>The plan card shows 'Trial · ends 5 Oct · 3 of 15 seats' with no way to upgrade. POST /api/billing/checkout (Razorpay) exists; no screen calls it.</t>
+        </is>
+      </c>
+      <c r="G393" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H393" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I393" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Needs Razorpay keys configured (billing_configured is false) and plan-picker UI.</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.52</t>
+        </is>
+      </c>
+      <c r="B394" s="28" t="inlineStr">
+        <is>
+          <t>Settings &gt; Account &gt; Password &amp; Security</t>
+        </is>
+      </c>
+      <c r="C394" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D394" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E394" s="28" t="inlineStr">
+        <is>
+          <t>Active sessions and sign out everywhere</t>
+        </is>
+      </c>
+      <c r="F394" s="28" t="inlineStr">
+        <is>
+          <t>GET/DELETE /api/auth/me/sessions exist; Settings offers only 'Sign out' of this device. A lost phone cannot be signed out from a laptop.</t>
+        </is>
+      </c>
+      <c r="G394" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H394" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I394" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Small: list sessions with device + last seen, sign out one / all others.</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.53</t>
+        </is>
+      </c>
+      <c r="B395" s="28" t="inlineStr">
+        <is>
+          <t>Settings &gt; Account</t>
+        </is>
+      </c>
+      <c r="C395" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D395" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E395" s="28" t="inlineStr">
+        <is>
+          <t>Notification preferences</t>
+        </is>
+      </c>
+      <c r="F395" s="28" t="inlineStr">
+        <is>
+          <t>No control over what reaches someone by email/WhatsApp/push; owners can only switch overdue-owner emails in Deadlines.</t>
+        </is>
+      </c>
+      <c r="G395" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H395" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I395" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Decide channels per event type (approvals, overdue, leave, mentions).</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.54</t>
+        </is>
+      </c>
+      <c r="B396" s="28" t="inlineStr">
+        <is>
+          <t>Settings &gt; Workspace</t>
+        </is>
+      </c>
+      <c r="C396" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D396" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E396" s="28" t="inlineStr">
+        <is>
+          <t>Owner self-serve export of company data</t>
+        </is>
+      </c>
+      <c r="F396" s="28" t="inlineStr">
+        <is>
+          <t>DPDP export exists only in the platform admin console; an owner cannot download their own company's data.</t>
+        </is>
+      </c>
+      <c r="G396" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H396" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I396" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Reuse the admin DSAR export, scoped to the owner's tenant.</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.55</t>
+        </is>
+      </c>
+      <c r="B397" s="28" t="inlineStr">
+        <is>
+          <t>Settings &gt; Business &gt; Company Details</t>
+        </is>
+      </c>
+      <c r="C397" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D397" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E397" s="28" t="inlineStr">
+        <is>
+          <t>Teams &amp; access deserve their own tab</t>
+        </is>
+      </c>
+      <c r="F397" s="28" t="inlineStr">
+        <is>
+          <t>Teams and their Access editor sit at the bottom of the Company Details card on the Business tab; owners look for them under Team or a 'Team &amp; access' tab.</t>
+        </is>
+      </c>
+      <c r="G397" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H397" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I397" s="28" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Design: move Teams + Access (and Leave approvers) to a 'Team &amp; access' tab, or link from the Team page.</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Settings: Team & access tab, two-pane desktop, access switches
- Team & access gets its own tab: teams + their access (TeamsCard), who
  approves leave, what owners can open. Task templates move to Operations.
  Company Details is only the company now.
- Desktop Settings is two panes: a sticky side panel (who you are, the
  sections, jump links to the cards on screen) beside the content column.
  Phone tabs scroll with whole labels and are real tabs.
- Members see what they can open (Your access).
- The remaining old square cards are restyled to the glass cards.
- Access areas are a light row with a switch (AccessSwitch) instead of
  tiles that turned solid black when on, in the team editor, the owner
  card and the member dialog.
- Scratch backend start script blanks every outbound messaging key in
  Python and refuses a non-scratch DB.

Tracker: U7-23.32..U7-23.61; Sprint 23 57/62. Full suite green
(2076 passed, 645 skipped).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 292 of 395 items Done  (74%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 50 of 56 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
+          <t>Epic 6 progress: 299 of 401 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 57 of 62 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2370,17 +2370,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>57</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>62</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L397"/>
+  <dimension ref="A1:L403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28448,17 +28448,359 @@
       </c>
       <c r="I397" s="28" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t>Design: move Teams + Access (and Leave approvers) to a 'Team &amp; access' tab, or link from the Team page.</t>
+          <t>SHIPPED 2026-10-05 (founder). Settings › Team &amp; access: Teams with their Access editor (components/settings/TeamsCard), Who approves leave (from Operations) and What owners can open (from Workspace). Head-count per team; delete disabled with a reason while a team has people; link to the Team page to add or move people. Task templates moved to Operations as their own card. Verified in the browser as owner: 6 tabs, all cards load, no failed requests.</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-03 (Settings product review + desktop pass, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.56</t>
+        </is>
+      </c>
+      <c r="B398" s="28" t="inlineStr">
+        <is>
+          <t>CompanyDetails, BusinessVocabulary, OperatingModelEditor, Leave approvers, RegenerateWithAi</t>
+        </is>
+      </c>
+      <c r="C398" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D398" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E398" s="28" t="inlineStr">
+        <is>
+          <t>Every Settings card in one style</t>
+        </is>
+      </c>
+      <c r="F398" s="28" t="inlineStr">
+        <is>
+          <t>Four cards were still on the old style — solid white tiles with square grey-bordered boxes and square UPPERCASE buttons — beside rounded glass cards on the same page (191 old borders on the Operating Model alone).</t>
+        </is>
+      </c>
+      <c r="G398" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H398" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I398" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. Glass card frame, glass fields, ink Save pills and glass secondary pills throughout; Company Details now only the company (fields, WhatsApp code, products) with one save. A computed-style sweep of all six tabs finds no old-style element left (the red Delete account is deliberate).</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (Settings UI/UX review, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.57</t>
+        </is>
+      </c>
+      <c r="B399" s="28" t="inlineStr">
+        <is>
+          <t>pages/Settings.js tab row</t>
+        </is>
+      </c>
+      <c r="C399" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D399" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E399" s="28" t="inlineStr">
+        <is>
+          <t>Settings tabs read whole on a phone</t>
+        </is>
+      </c>
+      <c r="F399" s="28" t="inlineStr">
+        <is>
+          <t>With six tabs each got 56px on a phone and the labels were cut ('Team &amp; a…', 'Operati…'). The row also said role=tablist while its buttons said aria-pressed.</t>
+        </is>
+      </c>
+      <c r="G399" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H399" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I399" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. Below lg the row scrolls with whole labels and brings the open tab into view; from lg up the tabs share the row. Buttons are role=tab with aria-selected.</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (Settings UI/UX review, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.58</t>
+        </is>
+      </c>
+      <c r="B400" s="28" t="inlineStr">
+        <is>
+          <t>pages/Settings.js YourAccessCard</t>
+        </is>
+      </c>
+      <c r="C400" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D400" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E400" s="28" t="inlineStr">
+        <is>
+          <t>A member can see what they can open</t>
+        </is>
+      </c>
+      <c r="F400" s="28" t="inlineStr">
+        <is>
+          <t>Nothing told a member what their access was; something missing might be access or a fault, and only the owner could say which.</t>
+        </is>
+      </c>
+      <c r="G400" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H400" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I400" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. Read-only 'Your access' card on a member's Settings (and a manager's Account tab), grouped like the editors, from the server-resolved list. Verified as Priya.</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (Settings UI/UX review, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.59</t>
+        </is>
+      </c>
+      <c r="B401" s="28" t="inlineStr">
+        <is>
+          <t>backend/scripts/run_scratch_backend.py; .claude/launch.json</t>
+        </is>
+      </c>
+      <c r="C401" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D401" s="28" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="E401" s="28" t="inlineStr">
+        <is>
+          <t>The scratch backend really has messaging off</t>
+        </is>
+      </c>
+      <c r="F401" s="28" t="inlineStr">
+        <is>
+          <t>The Windows launch entry blanked keys with cmd.exe `set NAME=`, which DELETES the variable; load_dotenv then refilled it from backend/.env with the live keys. DB stayed on the scratch database, but during this session's checks one login SMS went to the seeded number +91 98450 21921 and one owner-alert email to rajesh70595@kaveri-70595.in.</t>
+        </is>
+      </c>
+      <c r="G401" s="28" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H401" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I401" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. A Python start script sets every outbound key to EMPTY before the app loads (load_dotenv never overrides an existing variable) and refuses a non-scratch DB_NAME; both launch.json files use it. Verified: OTP request returns dev_mode true, sent false.</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (Settings UI/UX review, browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.60</t>
+        </is>
+      </c>
+      <c r="B402" s="28" t="inlineStr">
+        <is>
+          <t>pages/Settings.js SettingsShell / Section</t>
+        </is>
+      </c>
+      <c r="C402" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D402" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E402" s="28" t="inlineStr">
+        <is>
+          <t>Settings uses a desktop screen: two panes</t>
+        </is>
+      </c>
+      <c r="F402" s="28" t="inlineStr">
+        <is>
+          <t>On desktop Settings was one 600px column pinned to the left of a 1300px screen, the rest empty (founder screenshot: 'lot of space, no design').</t>
+        </is>
+      </c>
+      <c r="G402" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H402" s="28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I402" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. From lg up: a sticky side panel (who you are: name, team, company; then the sections — the owner's six tabs with a one-line description, the open tab listing its cards as jump links; a member's cards as jump links) beside a content column up to 52rem, centred. Links are read live from the cards on screen (MutationObserver; a card that renders nothing is never offered) and mark the card in view. Phone unchanged (tab row / single stack). Measured: 1366 side 252px + content 742px; 1024 side 230 + content 699; 1920 content ~1000; no horizontal scroll at 390/1024/1920.</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (screenshot of member Settings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.61</t>
+        </is>
+      </c>
+      <c r="B403" s="28" t="inlineStr">
+        <is>
+          <t>components/settings/AccessSwitch.js; TeamsCard.js; pages/Settings.js; pages/Team.js</t>
+        </is>
+      </c>
+      <c r="C403" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D403" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E403" s="28" t="inlineStr">
+        <is>
+          <t>Access is a switch, not a black tile</t>
+        </is>
+      </c>
+      <c r="F403" s="28" t="inlineStr">
+        <is>
+          <t>Every access area (team Access editor, What owners can open, the add/edit member dialog) was a tile that turned solid black when on; nearly every area IS on, so the cards were walls of black (founder screenshot: 'I don't like the black dark highlighting').</t>
+        </is>
+      </c>
+      <c r="G403" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H403" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I403" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. One shared AccessSwitch: a light row with the label and a switch in the app's primary colour (role=switch, aria-checked); an area that is off reads off (muted label, grey switch). Owners' Manage Team shows '· always on' and cannot be switched off. The member dialog's switches stay disabled while 'Use the team's access' is ticked. Menu preview chips and the open Access button moved from black to a light primary tint. Browser-checked: 19 switches per editor, toggles flip aria-checked and colour, no black tiles left.</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (screenshot of What owners can open)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Settings fits a phone: one pipeline open at a time, whole names, audit log
- Operating Model: each pipeline is a one-line summary (name, stages,
  tasks, stage path) that opens on tap, one at a time. At 390px the card
  went 8,443 -> 722px closed and Operations 12,076 -> 2,424px.
- Task category fields size to their name (were cut at 112px).
- Pipeline / category delete are tap targets.
- Audit log table loses its 32rem floor, so "Who" no longer hides behind
  a sideways scroll on a phone.
- Phone tab row has scroll padding so the open tab is not clipped by the
  row's rounded end.

Tracker: U7-23.62, U7-23.63; Sprint 23 59/64. Full suite green
(2080 passed, 645 skipped).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -1586,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 299 of 401 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 57 of 62 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
+          <t>Epic 6 progress: 301 of 403 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 59 of 64 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2370,12 +2370,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>59</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L403"/>
+  <dimension ref="A1:L405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28801,6 +28801,120 @@
       <c r="L403" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-05 (screenshot of What owners can open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.62</t>
+        </is>
+      </c>
+      <c r="B404" s="28" t="inlineStr">
+        <is>
+          <t>components/OperatingModelEditor.js</t>
+        </is>
+      </c>
+      <c r="C404" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D404" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E404" s="28" t="inlineStr">
+        <is>
+          <t>Operating Model: one pipeline open at a time; whole category names</t>
+        </is>
+      </c>
+      <c r="F404" s="28" t="inlineStr">
+        <is>
+          <t>On a phone the Operating Model card was 8,443px (~14 screens) because every pipeline showed every stage with every field, so Operations was 12,076px and Task templates / Deadlines sat below all of it. Task category fields were a fixed 112px, cutting 'Order Management' to 'Order Managen'.</t>
+        </is>
+      </c>
+      <c r="G404" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H404" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I404" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. Each pipeline is a one-line summary (name; N stages · N tasks · stage path) that opens on tap, one at a time; a lone pipeline starts open, a new one opens for its name. Category fields size to their name. Pipeline/category delete are tap targets. Measured at 390px: card 8,443 -&gt; 722px closed, Operations 12,076 -&gt; 2,424px; all 7 category names whole; no horizontal scroll.</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (check the settings page in mobile view)</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="28" t="inlineStr">
+        <is>
+          <t>U7-23.63</t>
+        </is>
+      </c>
+      <c r="B405" s="28" t="inlineStr">
+        <is>
+          <t>pages/Settings.js AuditLogCard; phone tab row</t>
+        </is>
+      </c>
+      <c r="C405" s="28" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D405" s="28" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="E405" s="28" t="inlineStr">
+        <is>
+          <t>Audit log and tab row fit a phone</t>
+        </is>
+      </c>
+      <c r="F405" s="28" t="inlineStr">
+        <is>
+          <t>The audit table had a 32rem floor, so on a phone 'Who' sat behind a sideways scroll (512px table in a 403px box). With Workspace open, the active pill was scrolled flush to the tab row's rounded end and clipped.</t>
+        </is>
+      </c>
+      <c r="G405" s="28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H405" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I405" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-10-05. Table floor removed (three short columns fit, text wraps); tab row has scroll padding so the open tab lands inside the row. Measured at 390px: audit box 403/403 (no scroll), open Workspace tab 3px inside the row end. Whole Settings checked at 390px on every owner tab: no horizontal scroll, last card clears the bottom bar.</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Yokesh 2026-10-05 (check the settings page in mobile view)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trackers: Requests becomes its own epic (Epic 11, new feature)
Founder 2026-10-21: a new feature gets its own epic. The 18 Requests tasks
move out of Epic 6 Sprint 26 into docs/DecisionOS_Epic11_Requests.xlsx
(Epic 9's layout), renumbered U7-26.x -> RQ-s.n with the old ID in Notes:
Sprint 1 backend 8/8, Sprint 2 web 6/6, Sprint 3 Phase 3 0/4.
Epic 6 is back to 301/403; the Master gains an Epic 11 row (913/1033).
REQUESTS_PLAN.md points at Epic 11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic6_UX_UI_Optimization.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B118"/>
+  <dimension ref="A1:B113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -644,7 +643,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -657,7 +655,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -670,7 +667,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -683,7 +679,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -691,7 +686,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
@@ -735,7 +729,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -779,7 +772,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
@@ -823,7 +815,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
@@ -867,7 +858,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
@@ -911,7 +901,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
@@ -955,7 +944,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
@@ -999,7 +987,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
@@ -1043,7 +1030,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
@@ -1087,7 +1073,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
@@ -1131,7 +1116,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
@@ -1175,7 +1159,6 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
@@ -1219,7 +1202,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
@@ -1263,7 +1245,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
@@ -1307,7 +1288,6 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
@@ -1351,7 +1331,6 @@
         </is>
       </c>
     </row>
-    <row r="89"/>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
@@ -1395,7 +1374,6 @@
         </is>
       </c>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
@@ -1439,7 +1417,6 @@
         </is>
       </c>
     </row>
-    <row r="99"/>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
@@ -1483,7 +1460,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
@@ -1527,7 +1503,6 @@
         </is>
       </c>
     </row>
-    <row r="109"/>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
@@ -1568,50 +1543,6 @@
       <c r="B113" t="inlineStr">
         <is>
           <t>In progress -- 12 of 13 Done; open: Phase 5 capture feedback</t>
-        </is>
-      </c>
-    </row>
-    <row r="114"/>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>Sprint 26 -- Requests (raise, approve, book the expense)</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Files</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>services/staff_requests.py, routers/staff_requests.py, components/requests/*, pages/Requests.js, pages/MyWork.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Employees had no way to ask for material, money or equipment and get a yes that reached Finance; it happened by word of mouth and the expense was typed again by hand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>In progress -- 14 of 18 Done; open: Phase 3 (voice via Dex, bill-photo reading, reports, WhatsApp)</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1655,7 +1586,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 315 of 421 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 59 of 64 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.  Sprint 26 (Requests) added 2026-10-21: 14 of 18 Done.</t>
+          <t>Epic 6 progress: 301 of 403 items Done  (75%).  7 items removed as obsolete after the karma redesign (logged with reasons in the 'Dropped (karma)' sheet).  UI rebuild recorded in the 'UI Redesign Log' sheet.  Backlog validated screen-by-screen vs the new UI on 2026-08-20.  Sprint 21 (My Work task management) added 2026-09-15: 14 of 16 Done.  Sprint 22 (Decision Desk decision flow) added 2026-09-15: 16 of 18 Done.  Sprint 23 (Settings, Team and access) added 2026-09-15: 59 of 64 Done.  Sprint 24 (Onboarding + auth) added 2026-09-17: 32 of 38 Done.  Sprint 25 (Workflows + tasks) added 2026-09-21: 80 of 88 Done.</t>
         </is>
       </c>
     </row>
@@ -2530,39 +2461,6 @@
       <c r="G30" t="inlineStr">
         <is>
           <t>Added 2026-09-21 after auditing the workflow + task sections from the Desk (docs/WORKFLOW_OPERATIONS_PLAN.md). The engine was real — stage gates, auto-advance, evidence, escalation — and the HUMAN half was missing: a person could not attach a task to a workflow, move a due date, repeat work or see more than one stage's slice. 19 items across continuity, control, visibility and continuous operations. A multi-user run (four people, two industries) found stage work going to nobody (departments never matched) — fixed — plus three findings for the founder. A 26-step walk by hand in the browser (3 people, real log-outs) fixed three more and logged the rest (docs/BROWSER_SCENARIOS_0921.md). The routines promised at sign-up are now confirmed once and repeat (U7-25.25). 2026-09-22: the workflow gets a clock — stage durations date the stage's work, stuck cards are reported, cards can carry a target date with a forecast, and the card shows planned vs actual per stage; the Desk's Delayed and Workflows tiles read it (U7-25.26–29).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Sprint 26</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Requests (raise, approve, book the expense)</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>14</v>
-      </c>
-      <c r="D31" t="n">
-        <v>18</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>78%</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Added 2026-10-21 from the client's Requests plan (docs/REQUESTS_PLAN.md): employees raise a request with one or many items, send it to their reporting manager (default) or the owner, approval books the expense in Finance, Finance marks it paid and purchases go into stock. Web first; Phase 3 (voice via Dex, bill-photo reading, reports, WhatsApp) is later. General requests are not financial: approval closes them, nothing goes to Finance.</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L423"/>
+  <dimension ref="A1:L405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -29017,996 +28915,6 @@
       <c r="L405" t="inlineStr">
         <is>
           <t>Yokesh 2026-10-05 (check the settings page in mobile view)</t>
-        </is>
-      </c>
-    </row>
-    <row r="406">
-      <c r="A406" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.1</t>
-        </is>
-      </c>
-      <c r="B406" s="28" t="inlineStr">
-        <is>
-          <t>services/staff_requests.py, models/staff_requests.py</t>
-        </is>
-      </c>
-      <c r="C406" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D406" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E406" s="28" t="inlineStr">
-        <is>
-          <t>The rules: seven types, approver choice, who may read / decide / fulfil</t>
-        </is>
-      </c>
-      <c r="F406" s="28" t="inlineStr">
-        <is>
-          <t>Types (Purchase &amp; materials, Expense reimbursement, Advance, Travel, Equipment &amp; assets, Repairs &amp; services, General) with their expense-category hint; approver = the requester's choice, reporting manager by default or the owner, no amount rule; no manager falls to the owner and says so; an owner's own request is recorded approved. Access: requester, approver or delegate, owner, Finance once approved; everyone else 404.</t>
-        </is>
-      </c>
-      <c r="G406" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H406" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I406" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K406" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L406" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="407">
-      <c r="A407" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.2</t>
-        </is>
-      </c>
-      <c r="B407" s="28" t="inlineStr">
-        <is>
-          <t>routers/staff_requests.py</t>
-        </is>
-      </c>
-      <c r="C407" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D407" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E407" s="28" t="inlineStr">
-        <is>
-          <t>The HTTP surface, every state change an atomic claim</t>
-        </is>
-      </c>
-      <c r="F407" s="28" t="inlineStr">
-        <is>
-          <t>GET /api/requests?view=mine|approvals|fulfil|all, GET approver-options, GET one; POST create, approve, reject (reason required), request-info, respond, withdraw, fulfil. Each update names the status it moves from, so two Approves make one approval and one expense; REQ-0001 numbering is one atomic increment per company with a unique index behind it.</t>
-        </is>
-      </c>
-      <c r="G407" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H407" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I407" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K407" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L407" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="408">
-      <c r="A408" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.3</t>
-        </is>
-      </c>
-      <c r="B408" s="28" t="inlineStr">
-        <is>
-          <t>routers/staff_requests.py _book_expense, routers/ledger.py create_expense</t>
-        </is>
-      </c>
-      <c r="C408" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D408" s="28" t="inlineStr">
-        <is>
-          <t>Requests / Finance</t>
-        </is>
-      </c>
-      <c r="E408" s="28" t="inlineStr">
-        <is>
-          <t>Approval books the expense in Finance</t>
-        </is>
-      </c>
-      <c r="F408" s="28" t="inlineStr">
-        <is>
-          <t>create_expense(source='request', request_id); the category is found in the company's own words (Raw Materials, Machine Maintenance) before the keyword guess; equipment books Asset Purchase so the asset register gets it; a reimbursement names the employee as payee. A failed booking keeps the approval and says so on the request.</t>
-        </is>
-      </c>
-      <c r="G408" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H408" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I408" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K408" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L408" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="409">
-      <c r="A409" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.4</t>
-        </is>
-      </c>
-      <c r="B409" s="28" t="inlineStr">
-        <is>
-          <t>routers/staff_requests.py fulfil, routers/ledger.py update_expense / delete_expense</t>
-        </is>
-      </c>
-      <c r="C409" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D409" s="28" t="inlineStr">
-        <is>
-          <t>Requests / Finance</t>
-        </is>
-      </c>
-      <c r="E409" s="28" t="inlineStr">
-        <is>
-          <t>Finance closes it: paid, and purchases into stock</t>
-        </is>
-      </c>
-      <c r="F409" s="28" t="inlineStr">
-        <is>
-          <t>Mark paid marks the booked expense paid and can put purchase items with a quantity into inventory (unit cost = line amount / quantity). Paying the expense in Finance closes the request on its own; deleting it unlinks the request and says why.</t>
-        </is>
-      </c>
-      <c r="G409" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H409" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I409" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K409" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L409" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="410">
-      <c r="A410" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.5</t>
-        </is>
-      </c>
-      <c r="B410" s="28" t="inlineStr">
-        <is>
-          <t>services/notifications.py, routers/staff_requests.py</t>
-        </is>
-      </c>
-      <c r="C410" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D410" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E410" s="28" t="inlineStr">
-        <is>
-          <t>Told at every step</t>
-        </is>
-      </c>
-      <c r="F410" s="28" t="inlineStr">
-        <is>
-          <t>Approver (and delegates) on a new request and an answer; requester on approve / reject / question / done; Finance and owners when something is approved to pay; approver when a request is withdrawn. Push titles: Request declined, Request withdrawn.</t>
-        </is>
-      </c>
-      <c r="G410" s="28" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H410" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I410" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K410" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L410" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="411">
-      <c r="A411" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.6</t>
-        </is>
-      </c>
-      <c r="B411" s="28" t="inlineStr">
-        <is>
-          <t>bootstrap/routing.py, bootstrap/lifecycle.py, services/tenant_wipe.py, routers/pulse.py, routers/files.py</t>
-        </is>
-      </c>
-      <c r="C411" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D411" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E411" s="28" t="inlineStr">
-        <is>
-          <t>Wired in on day one</t>
-        </is>
-      </c>
-      <c r="F411" s="28" t="inlineStr">
-        <is>
-          <t>Router registered; indexes (tenant+created, requester, approver+status, status, unique number); 'requests' in the tenant wipe list; pulse watches it; a bill attached to a request opens for whoever may open the request; read-gate inventory and API-parity baseline (+10 routes) updated.</t>
-        </is>
-      </c>
-      <c r="G411" s="28" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H411" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I411" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K411" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L411" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="412">
-      <c r="A412" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.7</t>
-        </is>
-      </c>
-      <c r="B412" s="28" t="inlineStr">
-        <is>
-          <t>tests/test_staff_requests.py, tests/fake_mongo.py</t>
-        </is>
-      </c>
-      <c r="C412" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D412" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E412" s="28" t="inlineStr">
-        <is>
-          <t>31 tests: routing, access, money, ask-back, attachments</t>
-        </is>
-      </c>
-      <c r="F412" s="28" t="inlineStr">
-        <is>
-          <t>Manager default / owner choice / no-manager fallback, numbering per company, validation, owner auto-record; access 404s, no self-approval, owner and delegate decide; one expense under two simultaneous approvals, failed booking keeps the yes, company categories, equipment asset, reimbursement payee, fulfil -&gt; paid + stock, expense paid -&gt; request done, delete unlinks; reject needs a reason, question/answer, withdraw rules; own-files-only attachments. FakeDB gains $push and find_one_and_update.</t>
-        </is>
-      </c>
-      <c r="G412" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H412" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I412" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K412" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L412" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="413">
-      <c r="A413" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.8</t>
-        </is>
-      </c>
-      <c r="B413" s="28" t="inlineStr">
-        <is>
-          <t>components/requests/NewWorkMenu.jsx, pages/MyWork.js, pages/Tasks.js</t>
-        </is>
-      </c>
-      <c r="C413" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D413" s="28" t="inlineStr">
-        <is>
-          <t>My Work</t>
-        </is>
-      </c>
-      <c r="E413" s="28" t="inlineStr">
-        <is>
-          <t>The + asks: New task or New request</t>
-        </is>
-      </c>
-      <c r="F413" s="28" t="inlineStr">
-        <is>
-          <t>My Work's + (phone circle and desktop '+ New') opens a glass menu with the two choices, the CRM add-menu pattern. NewTaskDialog gains a controlled mode (open / hideTrigger) so the menu can open it.</t>
-        </is>
-      </c>
-      <c r="G413" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H413" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I413" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K413" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L413" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.9</t>
-        </is>
-      </c>
-      <c r="B414" s="28" t="inlineStr">
-        <is>
-          <t>components/requests/NewRequestDialog.jsx, lib/requests.js</t>
-        </is>
-      </c>
-      <c r="C414" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D414" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E414" s="28" t="inlineStr">
-        <is>
-          <t>New request form</t>
-        </is>
-      </c>
-      <c r="F414" s="28" t="inlineStr">
-        <is>
-          <t>Type chips; many items with quantity / unit / amount and a live total; needed-by date; bill or photo attached; why it is needed; Send to: reporting manager (default) or owner, with the no-manager and owner-records-it cases said up front. Words kept as a draft. Same sheet shape as New Task.</t>
-        </is>
-      </c>
-      <c r="G414" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H414" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I414" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K414" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L414" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="415">
-      <c r="A415" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.10</t>
-        </is>
-      </c>
-      <c r="B415" s="28" t="inlineStr">
-        <is>
-          <t>components/requests/RequestCard.jsx</t>
-        </is>
-      </c>
-      <c r="C415" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D415" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E415" s="28" t="inlineStr">
-        <is>
-          <t>The request card</t>
-        </is>
-      </c>
-      <c r="F415" s="28" t="inlineStr">
-        <is>
-          <t>Status and type chips, number, total, items, reason, files, question and answer together, reject reason, where the money is (in Finance / paid / in stock / why not), history timeline; Approve / Reject / Ask, Send answer, Withdraw and Mark paid shown from the server's can-flags.</t>
-        </is>
-      </c>
-      <c r="G415" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H415" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I415" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K415" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L415" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="416">
-      <c r="A416" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.11</t>
-        </is>
-      </c>
-      <c r="B416" s="28" t="inlineStr">
-        <is>
-          <t>pages/Requests.js, components/requests/RequestsPanel.jsx, pages/MyWork.js</t>
-        </is>
-      </c>
-      <c r="C416" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D416" s="28" t="inlineStr">
-        <is>
-          <t>Requests / My Work</t>
-        </is>
-      </c>
-      <c r="E416" s="28" t="inlineStr">
-        <is>
-          <t>Requests page and My requests in My Work</t>
-        </is>
-      </c>
-      <c r="F416" s="28" t="inlineStr">
-        <is>
-          <t>/requests: Mine, To approve, To pay, All (owner), summary, ?tab= and ?request= deep links. My Work gets a 'My requests' view (phone view picker and desktop segment) with its own + New.</t>
-        </is>
-      </c>
-      <c r="G416" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H416" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I416" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K416" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L416" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.12</t>
-        </is>
-      </c>
-      <c r="B417" s="28" t="inlineStr">
-        <is>
-          <t>pages/MyWork.js approvals hub, pages/Desk.js</t>
-        </is>
-      </c>
-      <c r="C417" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D417" s="28" t="inlineStr">
-        <is>
-          <t>Approvals / Desk</t>
-        </is>
-      </c>
-      <c r="E417" s="28" t="inlineStr">
-        <is>
-          <t>Approvals hub Requests tab and a Desk card</t>
-        </is>
-      </c>
-      <c r="F417" s="28" t="inlineStr">
-        <is>
-          <t>Approvals gets a Requests tab beside Tasks and Leave, counted in the number on the way in; the Desk's Watch column shows a Requests card when something waits on you.</t>
-        </is>
-      </c>
-      <c r="G417" s="28" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H417" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I417" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K417" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L417" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="418">
-      <c r="A418" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.13</t>
-        </is>
-      </c>
-      <c r="B418" s="28" t="inlineStr">
-        <is>
-          <t>components/mobile/AllAppsPanel.jsx, lib/notif.js, hooks/usePulse.js, App.js</t>
-        </is>
-      </c>
-      <c r="C418" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D418" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E418" s="28" t="inlineStr">
-        <is>
-          <t>Phone More tile, notification links, live refresh</t>
-        </is>
-      </c>
-      <c r="F418" s="28" t="inlineStr">
-        <is>
-          <t>More -&gt; Requests; a request notification opens the approver's queue, Finance's list to pay or the requester's own list on the card; pulse refreshes requests, the Desk and expenses.</t>
-        </is>
-      </c>
-      <c r="G418" s="28" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H418" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I418" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K418" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L418" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="419">
-      <c r="A419" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.14</t>
-        </is>
-      </c>
-      <c r="B419" s="28" t="inlineStr">
-        <is>
-          <t>services/voice.py, Dex</t>
-        </is>
-      </c>
-      <c r="C419" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D419" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E419" s="28" t="inlineStr">
-        <is>
-          <t>Raise a request by voice through Dex</t>
-        </is>
-      </c>
-      <c r="F419" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3.</t>
-        </is>
-      </c>
-      <c r="G419" s="28" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H419" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I419" s="28" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="K419" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3 (later) per the client plan - not in this build</t>
-        </is>
-      </c>
-      <c r="L419" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="420">
-      <c r="A420" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.15</t>
-        </is>
-      </c>
-      <c r="B420" s="28" t="inlineStr">
-        <is>
-          <t>services/ingestion.py</t>
-        </is>
-      </c>
-      <c r="C420" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D420" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E420" s="28" t="inlineStr">
-        <is>
-          <t>Reimbursement read from a bill photo</t>
-        </is>
-      </c>
-      <c r="F420" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3: fill the items and amount from the photographed bill.</t>
-        </is>
-      </c>
-      <c r="G420" s="28" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H420" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I420" s="28" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="K420" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3 (later) per the client plan - not in this build</t>
-        </is>
-      </c>
-      <c r="L420" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.16</t>
-        </is>
-      </c>
-      <c r="B421" s="28" t="inlineStr">
-        <is>
-          <t>reports</t>
-        </is>
-      </c>
-      <c r="C421" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D421" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E421" s="28" t="inlineStr">
-        <is>
-          <t>Spend reports from requests</t>
-        </is>
-      </c>
-      <c r="F421" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3: who asked for what, approved and paid, by type and month.</t>
-        </is>
-      </c>
-      <c r="G421" s="28" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H421" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I421" s="28" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="K421" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3 (later) per the client plan - not in this build</t>
-        </is>
-      </c>
-      <c r="L421" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="422">
-      <c r="A422" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.17</t>
-        </is>
-      </c>
-      <c r="B422" s="28" t="inlineStr">
-        <is>
-          <t>services/whatsapp.py</t>
-        </is>
-      </c>
-      <c r="C422" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D422" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E422" s="28" t="inlineStr">
-        <is>
-          <t>Requests on WhatsApp</t>
-        </is>
-      </c>
-      <c r="F422" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3: raise and approve from WhatsApp.</t>
-        </is>
-      </c>
-      <c r="G422" s="28" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H422" s="28" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I422" s="28" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="K422" s="28" t="inlineStr">
-        <is>
-          <t>Phase 3 (later) per the client plan - not in this build</t>
-        </is>
-      </c>
-      <c r="L422" s="28" t="inlineStr">
-        <is>
-          <t>Client plan 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="423">
-      <c r="A423" s="28" t="inlineStr">
-        <is>
-          <t>U7-26.18</t>
-        </is>
-      </c>
-      <c r="B423" s="28" t="inlineStr">
-        <is>
-          <t>services/staff_requests.py goes_to_finance, routers/staff_requests.py, components/requests/*</t>
-        </is>
-      </c>
-      <c r="C423" s="28" t="n">
-        <v>26</v>
-      </c>
-      <c r="D423" s="28" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="E423" s="28" t="inlineStr">
-        <is>
-          <t>A General request is a yes, not money</t>
-        </is>
-      </c>
-      <c r="F423" s="28" t="inlineStr">
-        <is>
-          <t>Yokesh 2026-10-21: General is not financial. No amount on the form (any sent are dropped); approval closes it - no expense booked, Finance not told, never in To pay and cannot open it, Mark paid refused (409). The card reads 'Approved' and sits with the closed ones; the owner's own General request is recorded with no money. 3 tests.</t>
-        </is>
-      </c>
-      <c r="G423" s="28" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="H423" s="28" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I423" s="28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K423" s="28" t="inlineStr">
-        <is>
-          <t>Done 2026-10-21 (awaiting push). docs/REQUESTS_PLAN.md</t>
-        </is>
-      </c>
-      <c r="L423" s="28" t="inlineStr">
-        <is>
-          <t>Founder 2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>